<commit_message>
Apply polygon overlaps to grid; update site
Updates for WI model - application of polygon data to grids
Updated Reference files/Setup_data.xlsx
</commit_message>
<xml_diff>
--- a/Reference files/Setup_data.xlsx
+++ b/Reference files/Setup_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\HSM-and-mapping\Reference files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Levine\Documents\GitHub\HSM-and-mapping\Reference files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2EDAB2-B563-4F3F-A73B-8ABE7DE91CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24AD927F-FEC5-435E-86F5-5B8E50CB41A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ABA54846-BF8B-4CFF-808A-98E7C297F143}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{ABA54846-BF8B-4CFF-808A-98E7C297F143}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="5" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="164">
   <si>
     <t>Site</t>
   </si>
@@ -210,9 +210,6 @@
     <t>SL-South</t>
   </si>
   <si>
-    <t>Oysters in Florida GSI layer. Source FWC</t>
-  </si>
-  <si>
     <t>Description of data layer including source of data.</t>
   </si>
   <si>
@@ -490,6 +487,51 @@
   </si>
   <si>
     <t>Flow-salinity data</t>
+  </si>
+  <si>
+    <t>Model_column_name</t>
+  </si>
+  <si>
+    <t>Oyst</t>
+  </si>
+  <si>
+    <t>Sgrs</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Ala</t>
+  </si>
+  <si>
+    <t>Sha</t>
+  </si>
+  <si>
+    <t>Chnl</t>
+  </si>
+  <si>
+    <t>Buffers</t>
+  </si>
+  <si>
+    <t>Buff</t>
+  </si>
+  <si>
+    <t>Oyster_Buffers</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Buffer zones created using Oysters in Florida GIS layers</t>
+  </si>
+  <si>
+    <t>Oysters in Florida GIS layer. Source FWC</t>
+  </si>
+  <si>
+    <t>OYSTER</t>
   </si>
 </sst>
 </file>
@@ -624,7 +666,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2290EAFA-E702-4013-855B-8287C2917115}" name="Table1" displayName="Table1" ref="A1:D20" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2290EAFA-E702-4013-855B-8287C2917115}" name="Table1" displayName="Table1" ref="A1:D20" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A1:D20" xr:uid="{2290EAFA-E702-4013-855B-8287C2917115}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0F3EFAE7-C43F-43A4-98CD-33BD085FAA71}" name="Type"/>
@@ -637,7 +679,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E2821D4A-29BF-4DC8-B339-8E2AA5FC96D3}" name="Table2" displayName="Table2" ref="A1:D10" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E2821D4A-29BF-4DC8-B339-8E2AA5FC96D3}" name="Table2" displayName="Table2" ref="A1:D10" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:D10" xr:uid="{E2821D4A-29BF-4DC8-B339-8E2AA5FC96D3}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{6698C1C8-6642-4681-845E-5BC43253DE59}" name="Site"/>
@@ -650,12 +692,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6FA0BAA3-47DA-49C8-91CB-0A2E7355A2B5}" name="Table3" displayName="Table3" ref="A1:E9" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:E9" xr:uid="{6FA0BAA3-47DA-49C8-91CB-0A2E7355A2B5}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6FA0BAA3-47DA-49C8-91CB-0A2E7355A2B5}" name="Table3" displayName="Table3" ref="A1:F10" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:F10" xr:uid="{6FA0BAA3-47DA-49C8-91CB-0A2E7355A2B5}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{5519B2E3-398D-4910-B2B3-9C35C0C36B8E}" name="Parameter"/>
     <tableColumn id="2" xr3:uid="{89BFB1ED-5765-4484-8DD0-4EF9A48A6028}" name="Layer_name"/>
     <tableColumn id="5" xr3:uid="{3FC64101-BD91-46FF-93B8-B2B46BC9EF8F}" name="Column_name"/>
+    <tableColumn id="6" xr3:uid="{9BC23B7E-990C-4FCF-81C4-C9D6520A7BDE}" name="Model_column_name"/>
     <tableColumn id="3" xr3:uid="{D9807E9C-4BAF-484F-93F6-BF0E9DEB2EC4}" name="Priority"/>
     <tableColumn id="4" xr3:uid="{7C4466E1-8375-4529-8D01-8CEC01CDAA7D}" name="Description"/>
   </tableColumns>
@@ -1056,13 +1099,13 @@
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Z5" t="s">
         <v>52</v>
@@ -1138,13 +1181,13 @@
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.3">
@@ -1168,12 +1211,12 @@
         <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
         <v>23</v>
@@ -1200,25 +1243,25 @@
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1255,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1347,10 +1390,10 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
         <v>3</v>
@@ -1361,10 +1404,10 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D9" t="s">
         <v>3</v>
@@ -1375,10 +1418,10 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s">
         <v>3</v>
@@ -1389,10 +1432,10 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D11" t="s">
         <v>3</v>
@@ -1403,10 +1446,10 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
         <v>3</v>
@@ -1417,10 +1460,10 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
         <v>86</v>
-      </c>
-      <c r="C13" t="s">
-        <v>87</v>
       </c>
       <c r="D13" t="s">
         <v>3</v>
@@ -1431,10 +1474,10 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D14" t="s">
         <v>3</v>
@@ -1445,10 +1488,10 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" t="s">
         <v>127</v>
-      </c>
-      <c r="C15" t="s">
-        <v>128</v>
       </c>
       <c r="D15" t="s">
         <v>3</v>
@@ -1459,10 +1502,10 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16" t="s">
         <v>130</v>
-      </c>
-      <c r="C16" t="s">
-        <v>131</v>
       </c>
       <c r="D16" t="s">
         <v>3</v>
@@ -1473,10 +1516,10 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" t="s">
         <v>132</v>
-      </c>
-      <c r="C17" t="s">
-        <v>133</v>
       </c>
       <c r="D17" t="s">
         <v>49</v>
@@ -1487,10 +1530,10 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D18" t="s">
         <v>49</v>
@@ -1501,10 +1544,10 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D19" t="s">
         <v>49</v>
@@ -1515,10 +1558,10 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D20" t="s">
         <v>49</v>
@@ -1594,7 +1637,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1613,7 +1656,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5" t="s">
         <v>45</v>
@@ -1622,12 +1665,12 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -1636,12 +1679,12 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
@@ -1650,49 +1693,49 @@
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -1705,17 +1748,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EEC5A8C-2EDB-451C-AE63-50DA71E8941F}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" customWidth="1"/>
     <col min="2" max="2" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" customWidth="1"/>
-    <col min="5" max="5" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="21.33203125" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="6" max="6" width="36.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -1723,33 +1766,39 @@
         <v>24</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D2">
+        <v>163</v>
+      </c>
+      <c r="D2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E2">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1757,16 +1806,19 @@
         <v>21</v>
       </c>
       <c r="C3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
         <v>80</v>
       </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1774,98 +1826,136 @@
         <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4">
+        <v>79</v>
+      </c>
+      <c r="D4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4">
         <v>3</v>
       </c>
-      <c r="E4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5">
+        <v>75</v>
+      </c>
+      <c r="D5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5">
         <v>4</v>
       </c>
-      <c r="E5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" t="s">
         <v>77</v>
       </c>
-      <c r="D6">
-        <v>7</v>
-      </c>
-      <c r="E6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>156</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
         <v>71</v>
       </c>
-      <c r="C7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" t="s">
         <v>102</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>103</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
         <v>104</v>
       </c>
-      <c r="D8">
-        <v>8</v>
-      </c>
-      <c r="E8" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" t="s">
+        <v>153</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9" t="s">
         <v>148</v>
       </c>
-      <c r="B9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9">
-        <v>6</v>
-      </c>
-      <c r="E9" t="s">
-        <v>149</v>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -1895,10 +1985,10 @@
         <v>24</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1906,13 +1996,13 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1920,13 +2010,13 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1934,13 +2024,13 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1948,13 +2038,13 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1962,13 +2052,13 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1976,13 +2066,13 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1990,13 +2080,13 @@
         <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -2004,10 +2094,10 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" t="s">
         <v>14</v>
@@ -2018,10 +2108,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
         <v>15</v>
@@ -2032,10 +2122,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
         <v>17</v>
@@ -2046,10 +2136,10 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" t="s">
         <v>16</v>
@@ -2060,10 +2150,10 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
         <v>18</v>
@@ -2071,240 +2161,240 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" t="s">
         <v>102</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>103</v>
       </c>
-      <c r="C14" t="s">
-        <v>104</v>
-      </c>
       <c r="D14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" t="s">
         <v>102</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>103</v>
       </c>
-      <c r="C15" t="s">
-        <v>104</v>
-      </c>
       <c r="D15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D30" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -2315,10 +2405,10 @@
         <v>21</v>
       </c>
       <c r="C31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -2329,38 +2419,38 @@
         <v>22</v>
       </c>
       <c r="C32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B33" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D33" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B34" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C34" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update WQ configs for TB site & plotting optimizations
Minor updates for TB model.
Improved data joins (added lat/lon join
Added rasterization (ggrastr) and ragg device for faster/leaner map exports
Updated location_boundary to return a dataframe with Longitude/Latitude
Updated df join to limit to required columns and cast County to character
</commit_message>
<xml_diff>
--- a/Reference files/Setup_data.xlsx
+++ b/Reference files/Setup_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\HSM-and-mapping\Reference files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE9EEC6-83E9-4448-9CBD-3EC47344400C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF367EF-BD2D-44BA-9DC2-3F6C945451FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ABA54846-BF8B-4CFF-808A-98E7C297F143}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="223">
   <si>
     <t>Site</t>
   </si>
@@ -588,24 +588,6 @@
     <t>R</t>
   </si>
   <si>
-    <t>TB-Lower</t>
-  </si>
-  <si>
-    <t>TB-Middle</t>
-  </si>
-  <si>
-    <t>TB-Hillsborough</t>
-  </si>
-  <si>
-    <t>TB-Old</t>
-  </si>
-  <si>
-    <t>TB-Boca</t>
-  </si>
-  <si>
-    <t>TB-River</t>
-  </si>
-  <si>
     <t>CH</t>
   </si>
   <si>
@@ -640,18 +622,6 @@
   </si>
   <si>
     <t>W</t>
-  </si>
-  <si>
-    <t>CH-West</t>
-  </si>
-  <si>
-    <t>CH-Harbor</t>
-  </si>
-  <si>
-    <t>CH-Boca</t>
-  </si>
-  <si>
-    <t>CH-Pine</t>
   </si>
   <si>
     <t>SA</t>
@@ -1785,7 +1755,7 @@
         <v>169</v>
       </c>
       <c r="D21" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1799,7 +1769,7 @@
         <v>170</v>
       </c>
       <c r="D22" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1813,7 +1783,7 @@
         <v>171</v>
       </c>
       <c r="D23" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1827,7 +1797,7 @@
         <v>172</v>
       </c>
       <c r="D24" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1841,7 +1811,7 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1855,7 +1825,7 @@
         <v>174</v>
       </c>
       <c r="D26" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1869,7 +1839,7 @@
         <v>175</v>
       </c>
       <c r="D27" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1877,10 +1847,10 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C28" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D28" t="s">
         <v>3</v>
@@ -1891,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C29" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="D29" t="s">
         <v>3</v>
@@ -1905,10 +1875,10 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C30" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D30" t="s">
         <v>3</v>
@@ -1919,10 +1889,10 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C31" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D31" t="s">
         <v>3</v>
@@ -1933,10 +1903,10 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C32" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="D32" t="s">
         <v>3</v>
@@ -1947,10 +1917,10 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C33" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="D33" t="s">
         <v>3</v>
@@ -1961,10 +1931,10 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C34" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D34" t="s">
         <v>3</v>
@@ -1975,10 +1945,10 @@
         <v>1</v>
       </c>
       <c r="B35" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="C35" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="D35" t="s">
         <v>3</v>
@@ -1989,10 +1959,10 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="C36" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D36" t="s">
         <v>3</v>
@@ -2003,10 +1973,10 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C37" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D37" t="s">
         <v>3</v>
@@ -2017,10 +1987,10 @@
         <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="C38" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="D38" t="s">
         <v>3</v>
@@ -2031,13 +2001,13 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="C39" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="D39" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -2045,13 +2015,13 @@
         <v>1</v>
       </c>
       <c r="B40" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C40" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="D40" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -2059,13 +2029,13 @@
         <v>1</v>
       </c>
       <c r="B41" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="C41" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
@@ -2073,13 +2043,13 @@
         <v>1</v>
       </c>
       <c r="B42" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="C42" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="D42" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
@@ -2087,13 +2057,13 @@
         <v>1</v>
       </c>
       <c r="B43" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C43" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2278,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -2292,7 +2262,7 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>183</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -2306,7 +2276,7 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -2320,7 +2290,7 @@
         <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>185</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -2334,7 +2304,7 @@
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -2348,12 +2318,12 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B17" t="s">
         <v>178</v>
@@ -2362,12 +2332,12 @@
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>201</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B18" t="s">
         <v>180</v>
@@ -2376,40 +2346,40 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B19" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B20" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B21" t="s">
         <v>45</v>
@@ -2418,26 +2388,26 @@
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B22" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C22">
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B23" t="s">
         <v>3</v>
@@ -2446,40 +2416,40 @@
         <v>3</v>
       </c>
       <c r="D23" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B24" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C24">
         <v>4</v>
       </c>
       <c r="D24" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B25" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="C25">
         <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B26" t="s">
         <v>180</v>
@@ -2488,12 +2458,12 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B27" t="s">
         <v>45</v>
@@ -2502,26 +2472,26 @@
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B28" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C28">
         <v>3</v>
       </c>
       <c r="D28" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
@@ -2530,7 +2500,7 @@
         <v>4</v>
       </c>
       <c r="D29" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>